<commit_message>
Materiais: dado pessoal removido, estratificações, condutas e ata de reunião
- Termo de indicação de gestor/fiscal virou modelo em branco (tinha servidoras e matrículas)
- AVS e relatório de viagem sem CPF, conta e matrícula; estratificação de saúde mental sem a paciente
- Nomes de autor tirados das propriedades de todos os .docx/.xls/.xlsx
- Categorias novas: Estratificações de risco, Condutas clínicas
- Modelo de Ata de reunião com lista de presença e assinaturas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATERIAIS PUBLICADOS/RH E SERVIDOR/escala_setembro_2026.xlsx
+++ b/MATERIAIS PUBLICADOS/RH E SERVIDOR/escala_setembro_2026.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/da4a0fddad64b08f/Desktop/.claude apps/CentralDocumentos/MATERIAIS PUBLICADOS/RH E SERVIDOR/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_85DA8F955672829E621180974774E6BE559F864D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D88ACA34-9EE3-4879-8DA4-194177E45423}"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_85DA8F955672829E621180974774E6BE559F864D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FA48BFE-2BC4-43E6-80FC-2A25173C1B8D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="16220" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SETEMBRO" sheetId="1" r:id="rId1"/>
@@ -232,13 +227,22 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -246,15 +250,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -272,6 +267,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -563,16 +562,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AH22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="35" width="3.44140625" customWidth="1"/>
+    <col min="5" max="35" width="3.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:34" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16"/>
@@ -609,8 +608,8 @@
       <c r="AG1" s="16"/>
       <c r="AH1" s="16"/>
     </row>
-    <row r="2" spans="1:34" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:34" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="16"/>
@@ -647,14 +646,14 @@
       <c r="AG2" s="16"/>
       <c r="AH2" s="16"/>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A3" s="23" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="21" t="s">
         <v>3</v>
       </c>
       <c r="F3" s="16"/>
@@ -687,7 +686,7 @@
       <c r="AG3" s="16"/>
       <c r="AH3" s="16"/>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
       <c r="E4" s="2" t="s">
         <v>4</v>
       </c>
@@ -779,7 +778,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -883,7 +882,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:34" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -919,7 +918,7 @@
       <c r="AG6" s="8"/>
       <c r="AH6" s="8"/>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -955,7 +954,7 @@
       <c r="AG7" s="8"/>
       <c r="AH7" s="8"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A8" s="4"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -991,7 +990,7 @@
       <c r="AG8" s="8"/>
       <c r="AH8" s="8"/>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1027,7 +1026,7 @@
       <c r="AG9" s="8"/>
       <c r="AH9" s="8"/>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1063,7 +1062,7 @@
       <c r="AG10" s="8"/>
       <c r="AH10" s="8"/>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1099,7 +1098,7 @@
       <c r="AG11" s="8"/>
       <c r="AH11" s="8"/>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1135,7 +1134,7 @@
       <c r="AG12" s="8"/>
       <c r="AH12" s="8"/>
     </row>
-    <row r="13" spans="1:34" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:34" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1171,7 +1170,7 @@
       <c r="AG13" s="8"/>
       <c r="AH13" s="8"/>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1207,7 +1206,7 @@
       <c r="AG14" s="8"/>
       <c r="AH14" s="8"/>
     </row>
-    <row r="15" spans="1:34" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:34" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1243,9 +1242,9 @@
       <c r="AG15" s="8"/>
       <c r="AH15" s="8"/>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A17" s="9"/>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="16"/>
@@ -1253,7 +1252,7 @@
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="17" t="s">
+      <c r="I17" s="18" t="s">
         <v>13</v>
       </c>
       <c r="J17" s="16"/>
@@ -1261,7 +1260,7 @@
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
       <c r="O17" s="11"/>
-      <c r="P17" s="17" t="s">
+      <c r="P17" s="18" t="s">
         <v>14</v>
       </c>
       <c r="Q17" s="16"/>
@@ -1269,7 +1268,7 @@
       <c r="S17" s="16"/>
       <c r="T17" s="16"/>
       <c r="V17" s="12"/>
-      <c r="W17" s="17" t="s">
+      <c r="W17" s="18" t="s">
         <v>15</v>
       </c>
       <c r="X17" s="16"/>
@@ -1277,8 +1276,8 @@
       <c r="Z17" s="16"/>
       <c r="AA17" s="16"/>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A18" s="23" t="s">
+    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A18" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="16"/>
@@ -1315,8 +1314,8 @@
       <c r="AG18" s="16"/>
       <c r="AH18" s="16"/>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A19" s="18" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="16"/>
@@ -1353,8 +1352,8 @@
       <c r="AG19" s="16"/>
       <c r="AH19" s="16"/>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A21" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="16"/>
@@ -1391,8 +1390,8 @@
       <c r="AG21" s="16"/>
       <c r="AH21" s="16"/>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
+    <row r="22" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A22" s="17" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="16"/>

</xml_diff>